<commit_message>
CAN Bus Hub ver1.1
</commit_message>
<xml_diff>
--- a/CANBusHub/bom/CANBusHub.xlsx
+++ b/CANBusHub/bom/CANBusHub.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yugod\Documents\ロボット研究部\基板\Robocon2025-PCB\CANBusHub\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9C5715B-A9BC-4E87-8936-4ACE04C5BFAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69E62182-C0B0-4250-ABF2-6935F5A6A1B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{BD010420-876B-4347-99CD-E544F86399CC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BD010420-876B-4347-99CD-E544F86399CC}"/>
   </bookViews>
   <sheets>
     <sheet name="CANBusHub" sheetId="1" r:id="rId1"/>
@@ -1113,7 +1113,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A828B52-73EF-4790-862F-2F3770FA596F}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
@@ -1141,7 +1140,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1162,7 +1161,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1204,7 +1203,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -1225,7 +1224,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -1246,7 +1245,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -1267,7 +1266,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>23</v>
       </c>
@@ -1288,8 +1287,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.4"/>
-    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E10" s="1" t="s">
         <v>27</v>
       </c>
@@ -1301,7 +1299,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="E11" t="s">
         <v>29</v>
       </c>
@@ -1311,13 +1309,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="C1:C11" xr:uid="{7A828B52-73EF-4790-862F-2F3770FA596F}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="https://akizukidenshi.com/catalog/g/g105780/"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="C1:C11" xr:uid="{7A828B52-73EF-4790-862F-2F3770FA596F}"/>
   <phoneticPr fontId="18"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>